<commit_message>
(docs) modified percentual in planning file
</commit_message>
<xml_diff>
--- a/documentation/Planning-method.xlsx
+++ b/documentation/Planning-method.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="CALENDAR" sheetId="1" state="visible" r:id="rId3"/>
@@ -302,11 +302,10 @@
       <family val="2"/>
     </font>
     <font>
-      <b val="true"/>
       <i val="true"/>
-      <sz val="20"/>
+      <sz val="14"/>
       <color theme="0" tint="-0.5"/>
-      <name val="Aptos Narrow"/>
+      <name val="Aptos Display"/>
       <family val="0"/>
     </font>
     <font>
@@ -419,84 +418,80 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="19" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -601,7 +596,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1400" spc="-1" strike="noStrike">
+              <a:defRPr b="0" lang="pt-AO" sz="1400" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -609,7 +604,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr b="0" sz="1400" spc="-1" strike="noStrike">
+              <a:rPr b="0" lang="pt-AO" sz="1400" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
@@ -771,10 +766,10 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.158730158730159</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0.841269841269841</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -837,9 +832,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>360720</xdr:colOff>
+      <xdr:colOff>360360</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -847,8 +842,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6192360" y="590760"/>
-        <a:ext cx="5151960" cy="2742120"/>
+        <a:off x="6193080" y="590760"/>
+        <a:ext cx="5140080" cy="2741760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -860,26 +855,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>200160</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>152280</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>57240</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>19080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>151560</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>361800</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>104400</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="TextBox 4"/>
+        <xdr:cNvPr id="1" name="TextBox 2"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7758720" y="1295280"/>
-          <a:ext cx="2000880" cy="1341720"/>
+          <a:off x="8286840" y="1542960"/>
+          <a:ext cx="990360" cy="847440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -906,17 +901,17 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="1" i="1" lang="en-US" sz="2000" spc="-1" strike="noStrike">
+            <a:rPr b="0" i="1" lang="en-US" sz="1400" spc="-1" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="lt1">
                   <a:lumMod val="50000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:latin typeface="Aptos Narrow"/>
+              <a:latin typeface="Aptos Display"/>
             </a:rPr>
-            <a:t>1,3%</a:t>
+            <a:t>2,4%</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="pt-BR" sz="2000" spc="-1" strike="noStrike">
+          <a:endParaRPr b="0" lang="pt-BR" sz="1400" spc="-1" strike="noStrike">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1105,230 +1100,230 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8.43"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="9.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8.43"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="0" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="6" t="n">
         <v>46185</v>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="8" t="n">
         <f aca="false">SUM(Schedule!D3:D8)/COUNT(Schedule!D3:D8)</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="10" t="str">
+        <v>1</v>
+      </c>
+      <c r="F3" s="9" t="str">
         <f aca="false">IF(E3=0,$J$4,IF(E3&lt;1,$J$3,$J$2))</f>
-        <v>Peding</v>
-      </c>
-      <c r="G3" s="11" t="n">
+        <v>Completed</v>
+      </c>
+      <c r="G3" s="10" t="n">
         <f aca="false">(SUM(E3:E9)/COUNT(E3:E9))</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="11" t="n">
+        <v>0.158730158730159</v>
+      </c>
+      <c r="H3" s="10" t="n">
         <f aca="false">100%-(SUM(E3:E9)/COUNT(E3:E9))</f>
-        <v>1</v>
-      </c>
-      <c r="J3" s="12" t="s">
+        <v>0.841269841269841</v>
+      </c>
+      <c r="J3" s="11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="6" t="n">
         <f aca="false">B3+A3</f>
         <v>46195</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="8" t="n">
         <f aca="false">SUM(Schedule!D9:D17)/COUNT(Schedule!D9:D17)</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="str">
+        <v>0.111111111111111</v>
+      </c>
+      <c r="F4" s="12" t="str">
         <f aca="false">IF(E4=0,$J$4,IF(E4&lt;1,$J$3,$J$2))</f>
-        <v>Peding</v>
-      </c>
-      <c r="J4" s="14" t="s">
+        <v>In progress</v>
+      </c>
+      <c r="J4" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <f aca="false">B4+A4</f>
         <v>46215</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="8" t="n">
         <f aca="false">SUM(Schedule!D18:D18)/COUNT(Schedule!D18:D18)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="13" t="str">
+      <c r="F5" s="12" t="str">
         <f aca="false">IF(E5=0,$J$4,IF(E5&lt;1,$J$3,$J$2))</f>
         <v>Peding</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <f aca="false">B5+A5</f>
         <v>46220</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="8" t="n">
         <f aca="false">SUM(Schedule!D19:D39)/COUNT(Schedule!D19:D39)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="13" t="str">
+      <c r="F6" s="12" t="str">
         <f aca="false">IF(E6=0,$J$4,IF(E6&lt;1,$J$3,$J$2))</f>
         <v>Peding</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <f aca="false">B6+A6</f>
         <v>46245</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8" t="n">
         <f aca="false">SUM(Schedule!D40:D49)/COUNT(Schedule!D40:D49)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="13" t="str">
+      <c r="F7" s="12" t="str">
         <f aca="false">IF(E7=0,$J$4,IF(E7&lt;1,$J$3,$J$2))</f>
         <v>Peding</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <f aca="false">B7+A7</f>
         <v>46265</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="8" t="n">
         <f aca="false">SUM(Schedule!D50:D58)/COUNT(Schedule!D50:D58)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="13" t="str">
+      <c r="F8" s="12" t="str">
         <f aca="false">IF(E8=0,$J$4,IF(E8&lt;1,$J$3,$J$2))</f>
         <v>Peding</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <f aca="false">B8+A8</f>
         <v>46270</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="8" t="n">
         <f aca="false">SUM(Schedule!D59:D64)/COUNT(Schedule!D59:D64)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="13" t="str">
+      <c r="F9" s="12" t="str">
         <f aca="false">IF(E9=0,$J$4,IF(E9&lt;1,$J$3,$J$2))</f>
         <v>Peding</v>
       </c>
-      <c r="H9" s="15"/>
+      <c r="H9" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1362,1059 +1357,954 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D106"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="29.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="29.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="6.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="0" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="6" t="n">
         <v>46204</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="1" t="n">
-        <v>0</v>
+      <c r="D3" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="6" t="n">
         <v>46205</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="1" t="n">
-        <v>0</v>
+      <c r="D4" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>46206</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>0</v>
+      <c r="D5" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>46207</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>0</v>
+      <c r="D6" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>46208</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>0</v>
+      <c r="D7" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <v>46209</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>0</v>
+      <c r="D8" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>46210</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>0</v>
+      <c r="D9" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="6" t="n">
         <v>46211</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>46212</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>46213</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>46214</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="6" t="n">
         <v>46215</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>46216</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="6" t="n">
         <v>46217</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>46218</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="6" t="n">
         <v>46219</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="6" t="n">
         <v>46220</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="1" t="n">
+      <c r="C19" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="6" t="n">
         <v>46221</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="1" t="n">
+      <c r="C20" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="6" t="n">
         <v>46222</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" s="1" t="n">
+      <c r="C21" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="6" t="n">
         <v>46223</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D22" s="1" t="n">
+      <c r="C22" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="6" t="n">
         <v>46224</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="1" t="n">
+      <c r="C23" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="6" t="n">
         <v>46225</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" s="1" t="n">
+      <c r="C24" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="6" t="n">
         <v>46226</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" s="1" t="n">
+      <c r="C25" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="6" t="n">
         <v>46227</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D26" s="1" t="n">
+      <c r="C26" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D26" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="6" t="n">
         <v>46228</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D27" s="1" t="n">
+      <c r="C27" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="n">
+      <c r="A28" s="6" t="n">
         <v>46229</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D28" s="1" t="n">
+      <c r="C28" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="n">
+      <c r="A29" s="6" t="n">
         <v>46230</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" s="1" t="n">
+      <c r="C29" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="6" t="n">
         <v>46231</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D30" s="1" t="n">
+      <c r="C30" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D30" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="6" t="n">
         <v>46232</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" s="1" t="n">
+      <c r="C31" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D31" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="n">
+      <c r="A32" s="6" t="n">
         <v>46233</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C32" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D32" s="1" t="n">
+      <c r="C32" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D32" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="6" t="n">
         <v>46234</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C33" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D33" s="1" t="n">
+      <c r="C33" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="n">
+      <c r="A34" s="6" t="n">
         <v>46235</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="1" t="n">
+      <c r="C34" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="6" t="n">
         <v>46236</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" s="1" t="n">
+      <c r="C35" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="n">
+      <c r="A36" s="6" t="n">
         <v>46237</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D36" s="1" t="n">
+      <c r="C36" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D36" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="n">
+      <c r="A37" s="6" t="n">
         <v>46238</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D37" s="1" t="n">
+      <c r="C37" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D37" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="n">
+      <c r="A38" s="6" t="n">
         <v>46239</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C38" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D38" s="1" t="n">
+      <c r="C38" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D38" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="6" t="n">
         <v>46240</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D39" s="1" t="n">
+      <c r="C39" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D39" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="n">
+      <c r="A40" s="6" t="n">
         <v>46241</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C40" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D40" s="1" t="n">
+      <c r="C40" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D40" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="n">
+      <c r="A41" s="6" t="n">
         <v>46242</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C41" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D41" s="1" t="n">
+      <c r="C41" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D41" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="n">
+      <c r="A42" s="6" t="n">
         <v>46243</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D42" s="1" t="n">
+      <c r="C42" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D42" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="n">
+      <c r="A43" s="6" t="n">
         <v>46244</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C43" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D43" s="1" t="n">
+      <c r="C43" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D43" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="6" t="n">
         <v>46245</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C44" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D44" s="1" t="n">
+      <c r="C44" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="6" t="n">
         <v>46246</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C45" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D45" s="1" t="n">
+      <c r="C45" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D45" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="n">
+      <c r="A46" s="6" t="n">
         <v>46247</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C46" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D46" s="1" t="n">
+      <c r="C46" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D46" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="6" t="n">
         <v>46248</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C47" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D47" s="1" t="n">
+      <c r="C47" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D47" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="n">
+      <c r="A48" s="6" t="n">
         <v>46249</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C48" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D48" s="1" t="n">
+      <c r="C48" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D48" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="6" t="n">
         <v>46250</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C49" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D49" s="1" t="n">
+      <c r="C49" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D49" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="n">
+      <c r="A50" s="6" t="n">
         <v>46251</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C50" s="18" t="s">
+      <c r="C50" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D50" s="1" t="n">
+      <c r="D50" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="n">
+      <c r="A51" s="6" t="n">
         <v>46252</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="18" t="s">
+      <c r="C51" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D51" s="1" t="n">
+      <c r="D51" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="n">
+      <c r="A52" s="6" t="n">
         <v>46253</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="B52" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="18" t="s">
+      <c r="C52" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D52" s="1" t="n">
+      <c r="D52" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="n">
+      <c r="A53" s="6" t="n">
         <v>46254</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C53" s="18" t="s">
+      <c r="C53" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D53" s="1" t="n">
+      <c r="D53" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="n">
+      <c r="A54" s="6" t="n">
         <v>46255</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C54" s="18" t="s">
+      <c r="C54" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D54" s="1" t="n">
+      <c r="D54" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="n">
+      <c r="A55" s="6" t="n">
         <v>46256</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="B55" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C55" s="18" t="s">
+      <c r="C55" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D55" s="1" t="n">
+      <c r="D55" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="n">
+      <c r="A56" s="6" t="n">
         <v>46257</v>
       </c>
-      <c r="B56" s="8" t="s">
+      <c r="B56" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C56" s="18" t="s">
+      <c r="C56" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D56" s="1" t="n">
+      <c r="D56" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="n">
+      <c r="A57" s="6" t="n">
         <v>46258</v>
       </c>
-      <c r="B57" s="8" t="s">
+      <c r="B57" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C57" s="18" t="s">
+      <c r="C57" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D57" s="1" t="n">
+      <c r="D57" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="n">
+      <c r="A58" s="6" t="n">
         <v>46259</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="B58" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C58" s="18" t="s">
+      <c r="C58" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D58" s="1" t="n">
+      <c r="D58" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7" t="n">
+      <c r="A59" s="6" t="n">
         <v>46260</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C59" s="18" t="s">
+      <c r="C59" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="D59" s="1" t="n">
+      <c r="D59" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="7" t="n">
+      <c r="A60" s="6" t="n">
         <v>46261</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="B60" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C60" s="18" t="s">
+      <c r="C60" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="D60" s="1" t="n">
+      <c r="D60" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7" t="n">
+      <c r="A61" s="6" t="n">
         <v>46262</v>
       </c>
-      <c r="B61" s="8" t="s">
+      <c r="B61" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C61" s="18" t="s">
+      <c r="C61" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="D61" s="1" t="n">
+      <c r="D61" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="7" t="n">
+      <c r="A62" s="6" t="n">
         <v>46263</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B62" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C62" s="18" t="s">
+      <c r="C62" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D62" s="1" t="n">
+      <c r="D62" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="7" t="n">
+      <c r="A63" s="6" t="n">
         <v>46264</v>
       </c>
-      <c r="B63" s="8" t="s">
+      <c r="B63" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C63" s="18" t="s">
+      <c r="C63" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D63" s="1" t="n">
+      <c r="D63" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="7" t="n">
+      <c r="A64" s="6" t="n">
         <v>46265</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="B64" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C64" s="18" t="s">
+      <c r="C64" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="D64" s="1" t="n">
+      <c r="D64" s="0" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0"/>
-      <c r="B65" s="0"/>
-      <c r="C65" s="18"/>
-      <c r="D65" s="0"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0"/>
-      <c r="B66" s="0"/>
-      <c r="D66" s="0"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0"/>
-      <c r="B67" s="0"/>
-      <c r="D67" s="0"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0"/>
-      <c r="B68" s="0"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0"/>
-      <c r="B69" s="0"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0"/>
-      <c r="B70" s="0"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0"/>
-      <c r="B71" s="0"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0"/>
-      <c r="B72" s="0"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0"/>
-      <c r="B73" s="0"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0"/>
-      <c r="B74" s="0"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0"/>
-      <c r="B75" s="0"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0"/>
-      <c r="B76" s="0"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0"/>
-      <c r="B77" s="0"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0"/>
-      <c r="B78" s="0"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0"/>
-      <c r="B79" s="0"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0"/>
-      <c r="B80" s="0"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0"/>
-      <c r="B81" s="0"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0"/>
-      <c r="B82" s="0"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="0"/>
-      <c r="B83" s="0"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="0"/>
-      <c r="B84" s="0"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="0"/>
-      <c r="B85" s="0"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="0"/>
-      <c r="B86" s="0"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="0"/>
-      <c r="B87" s="0"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="0"/>
-      <c r="B88" s="0"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0"/>
-      <c r="B89" s="0"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="0"/>
-      <c r="B90" s="0"/>
+      <c r="C65" s="17"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="7"/>
+      <c r="A91" s="6"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="7"/>
+      <c r="A92" s="6"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="7"/>
+      <c r="A93" s="6"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="7"/>
+      <c r="A94" s="6"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="7"/>
+      <c r="A95" s="6"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="7"/>
+      <c r="A96" s="6"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="7"/>
+      <c r="A97" s="6"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="7"/>
+      <c r="A98" s="6"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="7"/>
+      <c r="A99" s="6"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="7"/>
+      <c r="A100" s="6"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="7"/>
+      <c r="A101" s="6"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="7"/>
+      <c r="A102" s="6"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="7"/>
+      <c r="A103" s="6"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="7"/>
+      <c r="A104" s="6"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="7"/>
+      <c r="A105" s="6"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="7"/>
+      <c r="A106" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2442,49 +2332,49 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="0" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="0" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="0" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>